<commit_message>
Drop Complete.measures from the Functional_traits deposit
Low-value column (specimen bookkeeping, not a trait). Removed from
03_FT_elev.R's deposit select(), from DataS1/Functional_traits.csv and
the working copy (column deletion only, values otherwise byte-identical),
from the Functional_traits sheet of Column_definitions_final.xlsx, and
from the column-name crosswalk (which also drops the already-stale
Source_elev row).

The xlsx also carries Aaron's in-progress pass over the AVONET trait
definitions.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DataS1/Column_definitions_final.xlsx
+++ b/DataS1/Column_definitions_final.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="312">
   <si>
     <t>Field_name</t>
   </si>
@@ -127,9 +127,6 @@
     <t>Total.individuals</t>
   </si>
   <si>
-    <t>See Tobias et al (2022)</t>
-  </si>
-  <si>
     <t>AVONET</t>
   </si>
   <si>
@@ -208,18 +205,12 @@
     <t>Migration_avo</t>
   </si>
   <si>
-    <t>Migratory status; see Tobias et al. 2022</t>
-  </si>
-  <si>
     <t>Sedentary, Partial, Long_distance</t>
   </si>
   <si>
     <t>Migration_bb</t>
   </si>
   <si>
-    <t>Migratory status; see Sekercioglu et al. (2025)</t>
-  </si>
-  <si>
     <t>BIRDBASE</t>
   </si>
   <si>
@@ -229,48 +220,27 @@
     <t>Primary_diet</t>
   </si>
   <si>
-    <t>Primary diet category; see Sekercioglu et al. (2025)</t>
-  </si>
-  <si>
     <t>Diet_breadth</t>
   </si>
   <si>
-    <t>Number of major food groups used; see Sekercioglu et al. (2025)</t>
-  </si>
-  <si>
     <t>Habitat_breadth</t>
   </si>
   <si>
-    <t>Number of major habitat types used; see Sekercioglu et al. (2025)</t>
-  </si>
-  <si>
     <t>Ecological_specialization</t>
   </si>
   <si>
-    <t>Ecological specialization index; see Sekercioglu et al. (2025)</t>
-  </si>
-  <si>
     <t>Higher = more specialized; max of 2 for a species using only one food group and one habitat type</t>
   </si>
   <si>
     <t>Clutch_min</t>
   </si>
   <si>
-    <t>Minimum clutch size; see Sekercioglu et al. (2025)</t>
-  </si>
-  <si>
     <t>Clutch_max</t>
   </si>
   <si>
-    <t>Maximum clutch size; see Sekercioglu et al. (2025)</t>
-  </si>
-  <si>
     <t>Clutch_mean</t>
   </si>
   <si>
-    <t>Mean of clutch_min and clutch_max; see Sekercioglu et al. (2025)</t>
-  </si>
-  <si>
     <t>Gen_length</t>
   </si>
   <si>
@@ -278,9 +248,6 @@
   </si>
   <si>
     <t>Elev_range</t>
-  </si>
-  <si>
-    <t>Elevational range width (Ayerbe-Quinones, 2018)</t>
   </si>
   <si>
     <t>Meters</t>
@@ -614,94 +581,406 @@
     <t>HBW/BirdLife checklist</t>
   </si>
   <si>
-    <t xml:space="preserve">Species name according to BirdLife International (HBW-BirdLife checklist v5, Dec 2020)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of specimens and live birds measured for the species</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of measured individuals with a complete set of morphometric measurements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beak length from the tip to the base of the skull (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beak length from the anterior edge of the nostrils to the tip (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beak width at the anterior edge of the nostrils (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beak depth at the anterior edge of the nostrils (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarsus length, from the notch between tibia and tarsus to the last scale at the bend of the foot (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wing length from the carpal joint (bend of the wing) to the tip of the longest primary, unflattened (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distance from the tip of the first secondary to the tip of the longest primary (mm); larger in more pointed wings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Length from the carpal joint to the tip of the outermost secondary (mm); roughly wing length minus Kipp's distance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 x Kipp's distance / wing length; index of wing pointedness and a proxy for dispersal ability</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distance from the tip of the longest rectrix to where the two central rectrices emerge from the skin (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Body mass (g), species mean across males and females</t>
+    <t>Number of measured individuals with a complete set of morphometric measurements</t>
+  </si>
+  <si>
+    <t>Predominant habitat type occupied by the species</t>
+  </si>
+  <si>
+    <t>Openness of the species' predominant habitat</t>
+  </si>
+  <si>
+    <t>Broad trophic category, assigned when one food type provides at least 70% of resources</t>
+  </si>
+  <si>
+    <t>Predominant resource used, assigned when it provides at least 60% of resources</t>
+  </si>
+  <si>
+    <t>Locomotion / foraging substrate the species uses most</t>
+  </si>
+  <si>
+    <t>Minimum latitude of the species' breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Maximum latitude of the species' breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Latitude of the geometric centre of the species' breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Longitude of the geometric centre of the species' breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Desert; Rock; Grassland; Shrubland; Woodland; Forest; Human Modified; Wetland; Riverine; Coastal; Marine</t>
+  </si>
+  <si>
+    <t>Dense (forest interior, thickets); Semi_open (open shrubland, parkland, thorn forest); Open (desert, grassland, open water, rocky habitat, cities, forest canopy)</t>
+  </si>
+  <si>
+    <t>Herbivore; Carnivore; Scavenger; Omnivore</t>
+  </si>
+  <si>
+    <t>Frugivore; Granivore; Nectarivore; Herbivore; Herbivore aquatic; Invertivore; Vertivore; Aquatic predator; Scavenger; Omnivore</t>
+  </si>
+  <si>
+    <t>Aerial (mostly in flight); Terrestrial (on the ground); Insessorial (perching above ground); Aquatic (on water); Generalist</t>
+  </si>
+  <si>
+    <t>Tarsus length (mm)</t>
+  </si>
+  <si>
+    <t>Unflattened wing length (mm)</t>
+  </si>
+  <si>
+    <t>Distance from the tip of the first secondary to the tip of the longest primary (mm)</t>
+  </si>
+  <si>
+    <t>Length from the carpal joint to the tip of the outermost secondary (mm)</t>
+  </si>
+  <si>
+    <t>100 x Kipp's distance / wing length</t>
+  </si>
+  <si>
+    <t>Tail length (mm)</t>
+  </si>
+  <si>
+    <t>Species mean mass (g) across sexes</t>
+  </si>
+  <si>
+    <t>Total area of the species' mapped breeding and resident range (km^2)</t>
+  </si>
+  <si>
+    <t>Migratory status AVONET</t>
+  </si>
+  <si>
+    <t>Migratory status BIRDBASE</t>
+  </si>
+  <si>
+    <t>Primary diet category</t>
+  </si>
+  <si>
+    <t>Number of major food groups used</t>
+  </si>
+  <si>
+    <t>Number of major habitat types used</t>
+  </si>
+  <si>
+    <t>Ecological specialization index</t>
+  </si>
+  <si>
+    <t>Minimum clutch size</t>
+  </si>
+  <si>
+    <t>Maximum clutch size</t>
+  </si>
+  <si>
+    <t>Mean of clutch_min and clutch_max</t>
+  </si>
+  <si>
+    <t>Elevational range width</t>
+  </si>
+  <si>
+    <t>Species name according to BirdLife International</t>
+  </si>
+  <si>
+    <t>From HBW-BirdLife checklist v5, Dec 2020</t>
+  </si>
+  <si>
+    <t>Number of individuals measured for the species</t>
+  </si>
+  <si>
+    <t>Length from base of the skull to tip of beak (mm)</t>
+  </si>
+  <si>
+    <t>Length from the anterior edge of the nostrils to the tip of beak (mm)</t>
+  </si>
+  <si>
+    <t>Width at the anterior edge of the nostrils (mm)</t>
+  </si>
+  <si>
+    <t>Depth at the anterior edge of the nostrils (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Field_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column_content_definition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Species_ayerbe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Species according to Ayerbe-Quiñones (2018)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayerbe-Quiñones (2018)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Species_bl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Species name according to BirdLife International</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVONET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From HBW-BirdLife checklist v5, Dec 2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total.individuals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of individuals measured for the species</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beak.Length_Culmen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Length from base of the skull to tip of beak (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beak.Length_Nares</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Length from the anterior edge of the nostrils to the tip of beak (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beak.Width</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Width at the anterior edge of the nostrils (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beak.Depth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depth at the anterior edge of the nostrils (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarsus.Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarsus length (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wing.Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unflattened wing length (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kipps.Distance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distance from the tip of the first secondary to the tip of the longest primary (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secondary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Length from the carpal joint to the tip of the outermost secondary (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hand-Wing.Index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 x Kipp's distance / wing length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tail.Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tail length (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Species mean mass (g) across sexes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Habitat</t>
   </si>
   <si>
     <t xml:space="preserve">Predominant habitat type occupied by the species</t>
   </si>
   <si>
+    <t xml:space="preserve">Desert; Rock; Grassland; Shrubland; Woodland; Forest; Human Modified; Wetland; Riverine; Coastal; Marine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Habitat.Density</t>
+  </si>
+  <si>
     <t xml:space="preserve">Openness of the species' predominant habitat</t>
   </si>
   <si>
+    <t xml:space="preserve">Dense (forest interior, thickets); Semi_open (open shrubland, parkland, thorn forest); Open (desert, grassland, open water, rocky habitat, cities, forest canopy)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trophic.Level</t>
+  </si>
+  <si>
     <t xml:space="preserve">Broad trophic category, assigned when one food type provides at least 70% of resources</t>
   </si>
   <si>
+    <t xml:space="preserve">Herbivore; Carnivore; Scavenger; Omnivore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trophic.Niche</t>
+  </si>
+  <si>
     <t xml:space="preserve">Predominant resource used, assigned when it provides at least 60% of resources</t>
   </si>
   <si>
+    <t xml:space="preserve">Frugivore; Granivore; Nectarivore; Herbivore; Herbivore aquatic; Invertivore; Vertivore; Aquatic predator; Scavenger; Omnivore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary.Lifestyle</t>
+  </si>
+  <si>
     <t xml:space="preserve">Locomotion / foraging substrate the species uses most</t>
   </si>
   <si>
+    <t xml:space="preserve">Aerial (mostly in flight); Terrestrial (on the ground); Insessorial (perching above ground); Aquatic (on water); Generalist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min.Latitude</t>
+  </si>
+  <si>
     <t xml:space="preserve">Minimum latitude of the species' breeding and resident range (decimal degrees)</t>
   </si>
   <si>
+    <t xml:space="preserve">Max.Latitude</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maximum latitude of the species' breeding and resident range (decimal degrees)</t>
   </si>
   <si>
+    <t xml:space="preserve">Centroid.Latitude</t>
+  </si>
+  <si>
     <t xml:space="preserve">Latitude of the geometric centre of the species' breeding and resident range (decimal degrees)</t>
   </si>
   <si>
+    <t xml:space="preserve">Centroid.Longitude</t>
+  </si>
+  <si>
     <t xml:space="preserve">Longitude of the geometric centre of the species' breeding and resident range (decimal degrees)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total area of the species' mapped breeding and resident range (km2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desert; Rock; Grassland; Shrubland; Woodland; Forest; Human Modified; Wetland; Riverine; Coastal; Marine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dense (forest interior, thickets); Semi_open (open shrubland, parkland, thorn forest); Open (desert, grassland, open water, rocky habitat, cities, forest canopy)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Herbivore; Carnivore; Scavenger; Omnivore</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frugivore; Granivore; Nectarivore; Herbivore; Herbivore aquatic; Invertivore; Vertivore; Aquatic predator; Scavenger; Omnivore</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aerial (mostly in flight); Terrestrial (on the ground); Insessorial (perching above ground); Aquatic (on water); Generalist</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Migratory behaviour of the species (three ordinal classes)</t>
+    <t xml:space="preserve">Range.Size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total area of the species' mapped breeding and resident range (km^2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forest_bin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whether AVONET's Habitat field is "Forest", "Woodland", or "Riverine"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Migration_avo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Migratory status AVONET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sedentary, Partial, Long_distance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Migration_bb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Migratory status BIRDBASE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIRDBASE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Migratory, Altitudinal, Irregular, Sedentary (species with no BIRDBASE record are assumed Sedentary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary_diet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary diet category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diet_breadth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of major food groups used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Habitat_breadth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of major habitat types used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ecological_specialization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ecological specialization index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Higher = more specialized; max of 2 for a species using only one food group and one habitat type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clutch_min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum clutch size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clutch_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum clutch size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clutch_mean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean of clutch_min and clutch_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gen_length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generation length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bird et al. 2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elev_range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elevational range width</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Iucn_red_list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IUCN Red List category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HBW/BirdLife checklist</t>
   </si>
 </sst>
 </file>
@@ -1052,37 +1331,37 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="B5" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6">
@@ -1090,45 +1369,45 @@
         <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="B7" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="B8" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="B10" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C10" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1158,240 +1437,240 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="B4" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="B6" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="B7" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="B8" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="C8" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="B9" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="B10" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="B11" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="B12" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="B13" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="B14" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="B15" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="B16" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="B17" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="B18" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B19" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="C19" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="B20" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="B21" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="C21" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="B22" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="B23" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="B24" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="C24" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="B25" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="C25" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="B26" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="C26" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B27" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="C27" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1421,120 +1700,120 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="B3" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="B4" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="B5" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="B6" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="B7" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="B8" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="B9" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="B10" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="C11" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="B12" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="C12" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="B13" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="B14" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="B15" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -1549,472 +1828,490 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="26.6640625" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="55.6640625" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="92.33203125" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="24.6640625" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="55.6640625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>218</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>219</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>220</v>
       </c>
       <c r="D1" t="s">
-        <v>30</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>222</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>223</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
-      </c>
+        <v>224</v>
+      </c>
+      <c r="D2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>225</v>
       </c>
       <c r="B3" t="s">
-        <v>189</v>
+        <v>226</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>227</v>
+      </c>
+      <c r="D3" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>229</v>
       </c>
       <c r="B4" t="s">
-        <v>190</v>
+        <v>230</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>231</v>
       </c>
       <c r="B5" t="s">
-        <v>191</v>
+        <v>232</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>233</v>
       </c>
       <c r="B6" t="s">
-        <v>192</v>
+        <v>234</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>235</v>
       </c>
       <c r="B7" t="s">
-        <v>193</v>
+        <v>236</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>237</v>
       </c>
       <c r="B8" t="s">
-        <v>194</v>
+        <v>238</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>239</v>
       </c>
       <c r="B9" t="s">
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>241</v>
       </c>
       <c r="B10" t="s">
-        <v>196</v>
+        <v>242</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>243</v>
       </c>
       <c r="B11" t="s">
-        <v>197</v>
+        <v>244</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>245</v>
       </c>
       <c r="B12" t="s">
-        <v>198</v>
+        <v>246</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>46</v>
+        <v>247</v>
       </c>
       <c r="B13" t="s">
-        <v>199</v>
+        <v>248</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>249</v>
       </c>
       <c r="B14" t="s">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>251</v>
       </c>
       <c r="B15" t="s">
-        <v>201</v>
+        <v>252</v>
       </c>
       <c r="C15" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>49</v>
+        <v>253</v>
       </c>
       <c r="B16" t="s">
-        <v>202</v>
+        <v>254</v>
       </c>
       <c r="C16" t="s">
-        <v>37</v>
+        <v>227</v>
+      </c>
+      <c r="D16" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>50</v>
+        <v>256</v>
       </c>
       <c r="B17" t="s">
-        <v>203</v>
+        <v>257</v>
       </c>
       <c r="C17" t="s">
-        <v>37</v>
+        <v>227</v>
       </c>
       <c r="D17" t="s">
-        <v>213</v>
+        <v>258</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>51</v>
+        <v>259</v>
       </c>
       <c r="B18" t="s">
-        <v>204</v>
+        <v>260</v>
       </c>
       <c r="C18" t="s">
-        <v>37</v>
+        <v>227</v>
       </c>
       <c r="D18" t="s">
-        <v>214</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>52</v>
+        <v>262</v>
       </c>
       <c r="B19" t="s">
-        <v>205</v>
+        <v>263</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>227</v>
       </c>
       <c r="D19" t="s">
-        <v>215</v>
+        <v>264</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>53</v>
+        <v>265</v>
       </c>
       <c r="B20" t="s">
-        <v>206</v>
+        <v>266</v>
       </c>
       <c r="C20" t="s">
-        <v>37</v>
+        <v>227</v>
       </c>
       <c r="D20" t="s">
-        <v>216</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>54</v>
+        <v>268</v>
       </c>
       <c r="B21" t="s">
-        <v>207</v>
+        <v>269</v>
       </c>
       <c r="C21" t="s">
-        <v>37</v>
-      </c>
-      <c r="D21" t="s">
-        <v>217</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D21"/>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>55</v>
+        <v>270</v>
       </c>
       <c r="B22" t="s">
-        <v>208</v>
+        <v>271</v>
       </c>
       <c r="C22" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D22"/>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>56</v>
+        <v>272</v>
       </c>
       <c r="B23" t="s">
-        <v>209</v>
+        <v>273</v>
       </c>
       <c r="C23" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D23"/>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>57</v>
+        <v>274</v>
       </c>
       <c r="B24" t="s">
-        <v>210</v>
+        <v>275</v>
       </c>
       <c r="C24" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D24"/>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>58</v>
+        <v>276</v>
       </c>
       <c r="B25" t="s">
-        <v>211</v>
+        <v>277</v>
       </c>
       <c r="C25" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D25"/>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>59</v>
+        <v>278</v>
       </c>
       <c r="B26" t="s">
-        <v>212</v>
+        <v>279</v>
       </c>
       <c r="C26" t="s">
-        <v>37</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D26"/>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>60</v>
+        <v>280</v>
       </c>
       <c r="B27" t="s">
-        <v>61</v>
+        <v>281</v>
       </c>
       <c r="C27" t="s">
-        <v>37</v>
+        <v>227</v>
+      </c>
+      <c r="D27" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>283</v>
       </c>
       <c r="B28" t="s">
-        <v>218</v>
+        <v>284</v>
       </c>
       <c r="C28" t="s">
-        <v>37</v>
+        <v>285</v>
       </c>
       <c r="D28" t="s">
-        <v>64</v>
+        <v>286</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>65</v>
+        <v>287</v>
       </c>
       <c r="B29" t="s">
-        <v>66</v>
+        <v>288</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
-      </c>
-      <c r="D29" t="s">
-        <v>68</v>
-      </c>
+        <v>285</v>
+      </c>
+      <c r="D29"/>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>69</v>
+        <v>289</v>
       </c>
       <c r="B30" t="s">
-        <v>70</v>
+        <v>290</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
-      </c>
+        <v>285</v>
+      </c>
+      <c r="D30"/>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>291</v>
       </c>
       <c r="B31" t="s">
-        <v>72</v>
+        <v>292</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
-      </c>
+        <v>285</v>
+      </c>
+      <c r="D31"/>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>73</v>
+        <v>293</v>
       </c>
       <c r="B32" t="s">
-        <v>74</v>
+        <v>294</v>
       </c>
       <c r="C32" t="s">
-        <v>67</v>
+        <v>285</v>
+      </c>
+      <c r="D32" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>75</v>
+        <v>296</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>297</v>
       </c>
       <c r="C33" t="s">
-        <v>67</v>
-      </c>
-      <c r="D33" t="s">
-        <v>77</v>
-      </c>
+        <v>285</v>
+      </c>
+      <c r="D33"/>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>78</v>
+        <v>298</v>
       </c>
       <c r="B34" t="s">
-        <v>79</v>
+        <v>299</v>
       </c>
       <c r="C34" t="s">
-        <v>67</v>
-      </c>
+        <v>285</v>
+      </c>
+      <c r="D34"/>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="B35" t="s">
-        <v>81</v>
+        <v>301</v>
       </c>
       <c r="C35" t="s">
-        <v>67</v>
-      </c>
+        <v>285</v>
+      </c>
+      <c r="D35"/>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>82</v>
+        <v>302</v>
       </c>
       <c r="B36" t="s">
-        <v>83</v>
+        <v>303</v>
       </c>
       <c r="C36" t="s">
-        <v>67</v>
+        <v>304</v>
+      </c>
+      <c r="D36" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>84</v>
+        <v>306</v>
       </c>
       <c r="B37" t="s">
-        <v>185</v>
+        <v>307</v>
       </c>
       <c r="C37" t="s">
-        <v>186</v>
+        <v>224</v>
       </c>
       <c r="D37" t="s">
-        <v>85</v>
+        <v>308</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>86</v>
+        <v>309</v>
       </c>
       <c r="B38" t="s">
-        <v>87</v>
+        <v>310</v>
       </c>
       <c r="C38" t="s">
-        <v>33</v>
-      </c>
-      <c r="D38" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="s">
-        <v>89</v>
-      </c>
-      <c r="B39" t="s">
-        <v>187</v>
-      </c>
-      <c r="C39" t="s">
-        <v>188</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="D38"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add Site_covs$N_visits; split Pc_length into span and duration
N_visits: surveys per location, the counterpart to Event_covs$N_reps.

Pc_length measured first-to-last-bird span, not survey duration. Now
Pc_obs_span (raw span, QA-only, dropped by 05) and Pc_duration
(deposit): CIPAV's measured span, a flat 10 minutes otherwise.
Event_covs and Site_covs column order follow the xlsx sheets.
</commit_message>
<xml_diff>
--- a/DataS1/Column_definitions_final.xlsx
+++ b/DataS1/Column_definitions_final.xlsx
@@ -1,23 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ubcca-my.sharepoint.com/personal/aaron_skinner2_ubc_ca/Documents/Academia/PhD/Analysis/Ssp-bird-data-wrangling/DataS1/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="74" documentId="11_2A7B806BDA388D21EAE73AD5D10BB879CF387425" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{912DDD6E-83BC-3045-BB39-7394314FFF0E}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="25120" windowHeight="14840" firstSheet="0" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="25120" windowHeight="14840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Bird_abundances" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Event_covs" sheetId="6" state="visible" r:id="rId2"/>
-    <sheet name="Site_covs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Functional_traits" sheetId="7" state="visible" r:id="rId4"/>
-    <sheet name="Taxonomy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Bird_abundances" sheetId="1" r:id="rId1"/>
+    <sheet name="Event_covs" sheetId="6" r:id="rId2"/>
+    <sheet name="Site_covs" sheetId="3" r:id="rId3"/>
+    <sheet name="Functional_traits" sheetId="7" r:id="rId4"/>
+    <sheet name="Taxonomy" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="218">
   <si>
     <t>Field_name</t>
   </si>
@@ -130,9 +137,6 @@
     <t>AVONET</t>
   </si>
   <si>
-    <t>Complete.measures</t>
-  </si>
-  <si>
     <t>Beak.Length_Culmen</t>
   </si>
   <si>
@@ -278,9 +282,6 @@
   </si>
   <si>
     <t>Start time of point count</t>
-  </si>
-  <si>
-    <t>Species Latin name according to Fernando Ayerbe's 2018 field guide (AOS-SACC)</t>
   </si>
   <si>
     <t>Count</t>
@@ -372,18 +373,12 @@
     <t>Julian date</t>
   </si>
   <si>
-    <t>Pc_length</t>
-  </si>
-  <si>
     <t>Length of point count</t>
   </si>
   <si>
     <t>N_samp_periods</t>
   </si>
   <si>
-    <t>Number of distinct 'Ano_grp's sampled</t>
-  </si>
-  <si>
     <t>N_reps</t>
   </si>
   <si>
@@ -393,13 +388,7 @@
     <t>Rep_year_grp</t>
   </si>
   <si>
-    <t>Point count repetition number within Ano_grp</t>
-  </si>
-  <si>
     <t>Rep_season</t>
-  </si>
-  <si>
-    <t>Point count repetition number within a season, where a season is defined as surveys conducted within 80 days.</t>
   </si>
   <si>
     <t>Spp_obs</t>
@@ -420,9 +409,6 @@
   </si>
   <si>
     <t>Weather</t>
-  </si>
-  <si>
-    <t>Weather categories standardized across datasets</t>
   </si>
   <si>
     <t>Despejado: Clear
@@ -446,9 +432,6 @@
     <t>Season</t>
   </si>
   <si>
-    <t>Whether the survey fell within the closed 80-day sampling window used elsewhere (see Rep_season), relative to the first survey of that Ano_grp</t>
-  </si>
-  <si>
     <t>Early = within 80 days of the first survey in that Ano_grp
 Late = 80+ days after</t>
   </si>
@@ -456,9 +439,6 @@
     <t>Sampling_day</t>
   </si>
   <si>
-    <t>Day number within a closed sampling period, counted from the first survey date at that institution/Ano_grp</t>
-  </si>
-  <si>
     <t>Day 1 = first survey date</t>
   </si>
   <si>
@@ -520,9 +500,6 @@
   </si>
   <si>
     <t>Tot_prec</t>
-  </si>
-  <si>
-    <t>Total annual precipitation in millimeters</t>
   </si>
   <si>
     <t>Predominant habitat within the 50 meter point count radius</t>
@@ -566,9 +543,6 @@
     <t>Distance_farm</t>
   </si>
   <si>
-    <t>Distance (m) from the point count to the nearest farm boundary, per the Sustainable Cattle Ranching project's farm polygons</t>
-  </si>
-  <si>
     <t>Generation length</t>
   </si>
   <si>
@@ -581,36 +555,6 @@
     <t>HBW/BirdLife checklist</t>
   </si>
   <si>
-    <t>Number of measured individuals with a complete set of morphometric measurements</t>
-  </si>
-  <si>
-    <t>Predominant habitat type occupied by the species</t>
-  </si>
-  <si>
-    <t>Openness of the species' predominant habitat</t>
-  </si>
-  <si>
-    <t>Broad trophic category, assigned when one food type provides at least 70% of resources</t>
-  </si>
-  <si>
-    <t>Predominant resource used, assigned when it provides at least 60% of resources</t>
-  </si>
-  <si>
-    <t>Locomotion / foraging substrate the species uses most</t>
-  </si>
-  <si>
-    <t>Minimum latitude of the species' breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
-    <t>Maximum latitude of the species' breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
-    <t>Latitude of the geometric centre of the species' breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
-    <t>Longitude of the geometric centre of the species' breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
     <t>Desert; Rock; Grassland; Shrubland; Woodland; Forest; Human Modified; Wetland; Riverine; Coastal; Marine</t>
   </si>
   <si>
@@ -632,12 +576,6 @@
     <t>Unflattened wing length (mm)</t>
   </si>
   <si>
-    <t>Distance from the tip of the first secondary to the tip of the longest primary (mm)</t>
-  </si>
-  <si>
-    <t>Length from the carpal joint to the tip of the outermost secondary (mm)</t>
-  </si>
-  <si>
     <t>100 x Kipp's distance / wing length</t>
   </si>
   <si>
@@ -647,9 +585,6 @@
     <t>Species mean mass (g) across sexes</t>
   </si>
   <si>
-    <t>Total area of the species' mapped breeding and resident range (km^2)</t>
-  </si>
-  <si>
     <t>Migratory status AVONET</t>
   </si>
   <si>
@@ -701,294 +636,83 @@
     <t>Depth at the anterior edge of the nostrils (mm)</t>
   </si>
   <si>
-    <t xml:space="preserve">Field_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Definition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Column_content_definition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Species_ayerbe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Species according to Ayerbe-Quiñones (2018)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ayerbe-Quiñones (2018)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Species_bl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Species name according to BirdLife International</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVONET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">From HBW-BirdLife checklist v5, Dec 2020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total.individuals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of individuals measured for the species</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beak.Length_Culmen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Length from base of the skull to tip of beak (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beak.Length_Nares</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Length from the anterior edge of the nostrils to the tip of beak (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beak.Width</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Width at the anterior edge of the nostrils (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beak.Depth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Depth at the anterior edge of the nostrils (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarsus.Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarsus length (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wing.Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unflattened wing length (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kipps.Distance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distance from the tip of the first secondary to the tip of the longest primary (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Secondary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Length from the carpal joint to the tip of the outermost secondary (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hand-Wing.Index</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 x Kipp's distance / wing length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tail.Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tail length (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Species mean mass (g) across sexes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Habitat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Predominant habitat type occupied by the species</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desert; Rock; Grassland; Shrubland; Woodland; Forest; Human Modified; Wetland; Riverine; Coastal; Marine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Habitat.Density</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Openness of the species' predominant habitat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dense (forest interior, thickets); Semi_open (open shrubland, parkland, thorn forest); Open (desert, grassland, open water, rocky habitat, cities, forest canopy)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trophic.Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Broad trophic category, assigned when one food type provides at least 70% of resources</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Herbivore; Carnivore; Scavenger; Omnivore</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trophic.Niche</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Predominant resource used, assigned when it provides at least 60% of resources</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frugivore; Granivore; Nectarivore; Herbivore; Herbivore aquatic; Invertivore; Vertivore; Aquatic predator; Scavenger; Omnivore</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Primary.Lifestyle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Locomotion / foraging substrate the species uses most</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aerial (mostly in flight); Terrestrial (on the ground); Insessorial (perching above ground); Aquatic (on water); Generalist</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Min.Latitude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minimum latitude of the species' breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Max.Latitude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maximum latitude of the species' breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Centroid.Latitude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latitude of the geometric centre of the species' breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Centroid.Longitude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Longitude of the geometric centre of the species' breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Range.Size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total area of the species' mapped breeding and resident range (km^2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forest_bin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Whether AVONET's Habitat field is "Forest", "Woodland", or "Riverine"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Migration_avo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Migratory status AVONET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sedentary, Partial, Long_distance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Migration_bb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Migratory status BIRDBASE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BIRDBASE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Migratory, Altitudinal, Irregular, Sedentary (species with no BIRDBASE record are assumed Sedentary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Primary_diet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Primary diet category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diet_breadth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of major food groups used</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Habitat_breadth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of major habitat types used</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ecological_specialization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ecological specialization index</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Higher = more specialized; max of 2 for a species using only one food group and one habitat type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clutch_min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minimum clutch size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clutch_max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maximum clutch size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clutch_mean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mean of clutch_min and clutch_max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gen_length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generation length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bird et al. 2020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Years</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elev_range</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elevational range width</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Iucn_red_list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IUCN Red List category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HBW/BirdLife checklist</t>
+    <t xml:space="preserve">Predominant habitat type occupied </t>
+  </si>
+  <si>
+    <t>Openness of predominant habitat</t>
+  </si>
+  <si>
+    <t>Broad trophic category</t>
+  </si>
+  <si>
+    <t>Predominant resource used</t>
+  </si>
+  <si>
+    <t>Predominant locomotion / foraging substrate</t>
+  </si>
+  <si>
+    <t>Minimum latitude of breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Maximum latitude of breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Area of breeding and resident range (km^2)</t>
+  </si>
+  <si>
+    <t>Distance from secondary1 to the longest primary (mm)</t>
+  </si>
+  <si>
+    <t>Length from carpal joint to tip of secondary1 (mm)</t>
+  </si>
+  <si>
+    <t>Latitude of centroid of breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Longitude of centroid of breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Species Latin name according to Ayerbe's 2018 field guide</t>
+  </si>
+  <si>
+    <t>Annual precipitation (millimeters)</t>
+  </si>
+  <si>
+    <t>Distance (m) from the point count to the nearest farm boundary</t>
+  </si>
+  <si>
+    <t>Pc_duration</t>
+  </si>
+  <si>
+    <t>Number of distinct 'Year_grp's sampled</t>
+  </si>
+  <si>
+    <t>Point count repetition number within Year_grp</t>
+  </si>
+  <si>
+    <t>Weather categories</t>
+  </si>
+  <si>
+    <t>Whether the survey fell within an 80-day sampling window relative to the first survey of that Year_grp</t>
+  </si>
+  <si>
+    <t>Point count repetition number within a season</t>
+  </si>
+  <si>
+    <t>Day number within a closed sampling period, per institution and Year_grp</t>
+  </si>
+  <si>
+    <t>N_visits</t>
+  </si>
+  <si>
+    <t>Total number of surveys at a point count location</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1314,11 +1038,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1329,85 +1056,85 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" t="s">
         <v>79</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>80</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>82</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>84</v>
       </c>
-      <c r="B4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>85</v>
       </c>
-      <c r="B5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="6">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>31</v>
       </c>
       <c r="B6" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>88</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>90</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
+      <c r="C9" t="s">
         <v>92</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>93</v>
       </c>
-      <c r="C9" t="s">
+      <c r="B10" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
+      <c r="C10" t="s">
         <v>95</v>
-      </c>
-      <c r="B10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C10" t="s">
-        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1417,14 +1144,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="129.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1435,242 +1163,242 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" t="s">
         <v>79</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>80</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>82</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
+      <c r="B7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>104</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B8" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
+      <c r="C8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B10" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>110</v>
+      </c>
+      <c r="B12" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>84</v>
       </c>
-      <c r="B7" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>106</v>
-      </c>
-      <c r="B8" t="s">
-        <v>107</v>
-      </c>
-      <c r="C8" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>109</v>
-      </c>
-      <c r="B9" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>110</v>
-      </c>
-      <c r="B10" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>111</v>
-      </c>
-      <c r="B11" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
+      <c r="B13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>209</v>
+      </c>
+      <c r="B14" t="s">
         <v>112</v>
       </c>
-      <c r="B12" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>85</v>
-      </c>
-      <c r="B13" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
+      <c r="B15" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>114</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B16" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>116</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B17" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B18" t="s">
+        <v>213</v>
+      </c>
+      <c r="C18" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s">
+      <c r="B19" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>118</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B20" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
+      <c r="C20" t="s">
         <v>120</v>
       </c>
-      <c r="B17" t="s">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
+      <c r="B21" t="s">
         <v>122</v>
       </c>
-      <c r="B18" t="s">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s">
+      <c r="B22" t="s">
+        <v>212</v>
+      </c>
+      <c r="C22" t="s">
         <v>124</v>
       </c>
-      <c r="B19" t="s">
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>125</v>
       </c>
-      <c r="C19" t="s">
+      <c r="B23" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
         <v>127</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B24" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="s">
-        <v>129</v>
-      </c>
-      <c r="B21" t="s">
-        <v>130</v>
-      </c>
-      <c r="C21" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
+      <c r="B25" t="s">
+        <v>215</v>
+      </c>
+      <c r="C25" t="s">
         <v>132</v>
       </c>
-      <c r="B22" t="s">
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
+      <c r="B26" t="s">
         <v>134</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C26" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>136</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B27" t="s">
         <v>137</v>
       </c>
-      <c r="C24" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s">
-        <v>139</v>
-      </c>
-      <c r="B25" t="s">
-        <v>140</v>
-      </c>
-      <c r="C25" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="s">
-        <v>142</v>
-      </c>
-      <c r="B26" t="s">
-        <v>143</v>
-      </c>
-      <c r="C26" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="s">
-        <v>145</v>
-      </c>
-      <c r="B27" t="s">
-        <v>146</v>
-      </c>
       <c r="C27" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1680,14 +1408,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="51.1640625" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="51.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1698,122 +1426,130 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" t="s">
         <v>82</v>
       </c>
-      <c r="B2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="3">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B3" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>144</v>
+      </c>
+      <c r="B6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B7" t="s">
         <v>147</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B8" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>160</v>
+      </c>
+      <c r="B9" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B10" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>216</v>
+      </c>
+      <c r="B11" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
+      <c r="B12" t="s">
         <v>149</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
+      <c r="B13" t="s">
         <v>151</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
+      <c r="B14" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" t="s">
         <v>153</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C15" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>155</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B16" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
+      <c r="C16" t="s">
         <v>157</v>
-      </c>
-      <c r="B8" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>159</v>
-      </c>
-      <c r="B9" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>161</v>
-      </c>
-      <c r="B10" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" t="s">
-        <v>163</v>
-      </c>
-      <c r="C11" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>165</v>
-      </c>
-      <c r="B12" t="s">
-        <v>166</v>
-      </c>
-      <c r="C12" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>168</v>
-      </c>
-      <c r="B13" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>170</v>
-      </c>
-      <c r="B14" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>172</v>
-      </c>
-      <c r="B15" t="s">
-        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -1823,495 +1559,469 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:D38"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.6640625" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="92.33203125" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="55.6640625" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" customWidth="1"/>
+    <col min="2" max="2" width="92.33203125" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="55.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>218</v>
+        <v>27</v>
       </c>
       <c r="B1" t="s">
-        <v>219</v>
+        <v>28</v>
       </c>
       <c r="C1" t="s">
-        <v>220</v>
+        <v>29</v>
       </c>
       <c r="D1" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>222</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>223</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>224</v>
-      </c>
-      <c r="D2"/>
-    </row>
-    <row r="3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>225</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>226</v>
+        <v>187</v>
       </c>
       <c r="C3" t="s">
-        <v>227</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>229</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="C4" t="s">
-        <v>227</v>
-      </c>
-      <c r="D4"/>
-    </row>
-    <row r="5">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>231</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>232</v>
+        <v>190</v>
       </c>
       <c r="C5" t="s">
-        <v>227</v>
-      </c>
-      <c r="D5"/>
-    </row>
-    <row r="6">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>233</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>234</v>
+        <v>191</v>
       </c>
       <c r="C6" t="s">
-        <v>227</v>
-      </c>
-      <c r="D6"/>
-    </row>
-    <row r="7">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>235</v>
+        <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>236</v>
+        <v>192</v>
       </c>
       <c r="C7" t="s">
-        <v>227</v>
-      </c>
-      <c r="D7"/>
-    </row>
-    <row r="8">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>237</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>238</v>
+        <v>193</v>
       </c>
       <c r="C8" t="s">
-        <v>227</v>
-      </c>
-      <c r="D8"/>
-    </row>
-    <row r="9">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>239</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>240</v>
+        <v>172</v>
       </c>
       <c r="C9" t="s">
-        <v>227</v>
-      </c>
-      <c r="D9"/>
-    </row>
-    <row r="10">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>241</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>242</v>
+        <v>173</v>
       </c>
       <c r="C10" t="s">
-        <v>227</v>
-      </c>
-      <c r="D10"/>
-    </row>
-    <row r="11">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>243</v>
+        <v>43</v>
       </c>
       <c r="B11" t="s">
-        <v>244</v>
+        <v>202</v>
       </c>
       <c r="C11" t="s">
-        <v>227</v>
-      </c>
-      <c r="D11"/>
-    </row>
-    <row r="12">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>245</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>246</v>
+        <v>203</v>
       </c>
       <c r="C12" t="s">
-        <v>227</v>
-      </c>
-      <c r="D12"/>
-    </row>
-    <row r="13">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>247</v>
+        <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>248</v>
+        <v>174</v>
       </c>
       <c r="C13" t="s">
-        <v>227</v>
-      </c>
-      <c r="D13"/>
-    </row>
-    <row r="14">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>249</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="C14" t="s">
-        <v>227</v>
-      </c>
-      <c r="D14"/>
-    </row>
-    <row r="15">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>251</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>252</v>
+        <v>176</v>
       </c>
       <c r="C15" t="s">
-        <v>227</v>
-      </c>
-      <c r="D15"/>
-    </row>
-    <row r="16">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>253</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>254</v>
+        <v>194</v>
       </c>
       <c r="C16" t="s">
-        <v>227</v>
+        <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>256</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s">
-        <v>257</v>
+        <v>195</v>
       </c>
       <c r="C17" t="s">
-        <v>227</v>
+        <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>259</v>
+        <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>260</v>
+        <v>196</v>
       </c>
       <c r="C18" t="s">
-        <v>227</v>
+        <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>262</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>263</v>
+        <v>197</v>
       </c>
       <c r="C19" t="s">
-        <v>227</v>
+        <v>36</v>
       </c>
       <c r="D19" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>265</v>
+        <v>52</v>
       </c>
       <c r="B20" t="s">
-        <v>266</v>
+        <v>198</v>
       </c>
       <c r="C20" t="s">
-        <v>227</v>
+        <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>268</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>269</v>
+        <v>199</v>
       </c>
       <c r="C21" t="s">
-        <v>227</v>
-      </c>
-      <c r="D21"/>
-    </row>
-    <row r="22">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>270</v>
+        <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>271</v>
+        <v>200</v>
       </c>
       <c r="C22" t="s">
-        <v>227</v>
-      </c>
-      <c r="D22"/>
-    </row>
-    <row r="23">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>272</v>
+        <v>55</v>
       </c>
       <c r="B23" t="s">
-        <v>273</v>
+        <v>204</v>
       </c>
       <c r="C23" t="s">
-        <v>227</v>
-      </c>
-      <c r="D23"/>
-    </row>
-    <row r="24">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>274</v>
+        <v>56</v>
       </c>
       <c r="B24" t="s">
-        <v>275</v>
+        <v>205</v>
       </c>
       <c r="C24" t="s">
-        <v>227</v>
-      </c>
-      <c r="D24"/>
-    </row>
-    <row r="25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>276</v>
+        <v>57</v>
       </c>
       <c r="B25" t="s">
-        <v>277</v>
+        <v>201</v>
       </c>
       <c r="C25" t="s">
-        <v>227</v>
-      </c>
-      <c r="D25"/>
-    </row>
-    <row r="26">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>278</v>
+        <v>58</v>
       </c>
       <c r="B26" t="s">
-        <v>279</v>
+        <v>59</v>
       </c>
       <c r="C26" t="s">
-        <v>227</v>
-      </c>
-      <c r="D26"/>
-    </row>
-    <row r="27">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>280</v>
+        <v>60</v>
       </c>
       <c r="B27" t="s">
-        <v>281</v>
+        <v>177</v>
       </c>
       <c r="C27" t="s">
-        <v>227</v>
+        <v>36</v>
       </c>
       <c r="D27" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="28">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>283</v>
+        <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>284</v>
+        <v>178</v>
       </c>
       <c r="C28" t="s">
-        <v>285</v>
+        <v>63</v>
       </c>
       <c r="D28" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>287</v>
+        <v>65</v>
       </c>
       <c r="B29" t="s">
-        <v>288</v>
+        <v>179</v>
       </c>
       <c r="C29" t="s">
-        <v>285</v>
-      </c>
-      <c r="D29"/>
-    </row>
-    <row r="30">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>289</v>
+        <v>66</v>
       </c>
       <c r="B30" t="s">
-        <v>290</v>
+        <v>180</v>
       </c>
       <c r="C30" t="s">
-        <v>285</v>
-      </c>
-      <c r="D30"/>
-    </row>
-    <row r="31">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>291</v>
+        <v>67</v>
       </c>
       <c r="B31" t="s">
-        <v>292</v>
+        <v>181</v>
       </c>
       <c r="C31" t="s">
-        <v>285</v>
-      </c>
-      <c r="D31"/>
-    </row>
-    <row r="32">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>293</v>
+        <v>68</v>
       </c>
       <c r="B32" t="s">
-        <v>294</v>
+        <v>182</v>
       </c>
       <c r="C32" t="s">
-        <v>285</v>
+        <v>63</v>
       </c>
       <c r="D32" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>296</v>
+        <v>70</v>
       </c>
       <c r="B33" t="s">
-        <v>297</v>
+        <v>183</v>
       </c>
       <c r="C33" t="s">
-        <v>285</v>
-      </c>
-      <c r="D33"/>
-    </row>
-    <row r="34">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>298</v>
+        <v>71</v>
       </c>
       <c r="B34" t="s">
-        <v>299</v>
+        <v>184</v>
       </c>
       <c r="C34" t="s">
-        <v>285</v>
-      </c>
-      <c r="D34"/>
-    </row>
-    <row r="35">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>300</v>
+        <v>72</v>
       </c>
       <c r="B35" t="s">
-        <v>301</v>
+        <v>185</v>
       </c>
       <c r="C35" t="s">
-        <v>285</v>
-      </c>
-      <c r="D35"/>
-    </row>
-    <row r="36">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>302</v>
+        <v>73</v>
       </c>
       <c r="B36" t="s">
-        <v>303</v>
+        <v>163</v>
       </c>
       <c r="C36" t="s">
-        <v>304</v>
+        <v>164</v>
       </c>
       <c r="D36" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="37">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>306</v>
+        <v>75</v>
       </c>
       <c r="B37" t="s">
-        <v>307</v>
+        <v>186</v>
       </c>
       <c r="C37" t="s">
-        <v>224</v>
+        <v>33</v>
       </c>
       <c r="D37" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="38">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>309</v>
+        <v>77</v>
       </c>
       <c r="B38" t="s">
-        <v>310</v>
+        <v>165</v>
       </c>
       <c r="C38" t="s">
-        <v>311</v>
-      </c>
-      <c r="D38"/>
+        <v>166</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2320,11 +2030,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2335,7 +2045,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2343,7 +2053,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -2351,7 +2061,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2359,7 +2069,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2367,7 +2077,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2375,7 +2085,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -2383,7 +2093,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -2391,7 +2101,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -2399,7 +2109,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -2407,7 +2117,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -2415,7 +2125,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -2423,7 +2133,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>25</v>
       </c>

</xml_diff>

<commit_message>
Column definitions: fix the canopy-buffer descriptions
</commit_message>
<xml_diff>
--- a/DataS1/Column_definitions_final.xlsx
+++ b/DataS1/Column_definitions_final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ubcca-my.sharepoint.com/personal/aaron_skinner2_ubc_ca/Documents/Academia/PhD/Analysis/Ssp-bird-data-wrangling/DataS1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="11_2A7B806BDA388D21EAE73AD5D10BB879CF387425" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{912DDD6E-83BC-3045-BB39-7394314FFF0E}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="11_2A7B806BDA388D21EAE73AD5D10BB879CF387425" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D942B36-CE6E-6646-9D07-396AC5BCF946}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="25120" windowHeight="14840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="25120" windowHeight="14840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bird_abundances" sheetId="1" r:id="rId1"/>
@@ -445,16 +445,10 @@
     <t>Canopy_cover</t>
   </si>
   <si>
-    <t>Percent canopy cover within a 1 km buffer, see Popatov et al. (2026)</t>
-  </si>
-  <si>
     <t>0-100%</t>
   </si>
   <si>
     <t>Canopy_height_m</t>
-  </si>
-  <si>
-    <t>Canopy height (in meters) within the point count buffer, see Popatov et al. (2026)</t>
   </si>
   <si>
     <t>Id_scr</t>
@@ -706,6 +700,12 @@
   </si>
   <si>
     <t>Total number of surveys at a point count location</t>
+  </si>
+  <si>
+    <t>Percent canopy cover within a 1 km buffer, see Potapov et al. (2026)</t>
+  </si>
+  <si>
+    <t>Max canopy height (in meters) within the point count buffer, see Potapov et al. (2026)</t>
   </si>
 </sst>
 </file>
@@ -1096,7 +1096,7 @@
         <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -1273,7 +1273,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B14" t="s">
         <v>112</v>
@@ -1284,7 +1284,7 @@
         <v>113</v>
       </c>
       <c r="B15" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -1300,7 +1300,7 @@
         <v>116</v>
       </c>
       <c r="B17" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -1308,7 +1308,7 @@
         <v>129</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C18" t="s">
         <v>130</v>
@@ -1319,7 +1319,7 @@
         <v>117</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -1346,7 +1346,7 @@
         <v>123</v>
       </c>
       <c r="B22" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C22" t="s">
         <v>124</v>
@@ -1373,7 +1373,7 @@
         <v>131</v>
       </c>
       <c r="B25" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C25" t="s">
         <v>132</v>
@@ -1384,18 +1384,18 @@
         <v>133</v>
       </c>
       <c r="B26" t="s">
+        <v>216</v>
+      </c>
+      <c r="C26" t="s">
         <v>134</v>
-      </c>
-      <c r="C26" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B27" t="s">
-        <v>137</v>
+        <v>217</v>
       </c>
       <c r="C27" t="s">
         <v>76</v>
@@ -1436,98 +1436,98 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B7" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B9" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B10" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B11" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B12" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B13" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B14" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -1535,21 +1535,21 @@
         <v>48</v>
       </c>
       <c r="B15" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C15" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>153</v>
+      </c>
+      <c r="B16" t="s">
+        <v>154</v>
+      </c>
+      <c r="C16" t="s">
         <v>155</v>
-      </c>
-      <c r="B16" t="s">
-        <v>156</v>
-      </c>
-      <c r="C16" t="s">
-        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -1599,13 +1599,13 @@
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C3" t="s">
         <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -1613,7 +1613,7 @@
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C4" t="s">
         <v>36</v>
@@ -1624,7 +1624,7 @@
         <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
@@ -1635,7 +1635,7 @@
         <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C6" t="s">
         <v>36</v>
@@ -1646,7 +1646,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
@@ -1657,7 +1657,7 @@
         <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C8" t="s">
         <v>36</v>
@@ -1668,7 +1668,7 @@
         <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C9" t="s">
         <v>36</v>
@@ -1679,7 +1679,7 @@
         <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C10" t="s">
         <v>36</v>
@@ -1690,7 +1690,7 @@
         <v>43</v>
       </c>
       <c r="B11" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -1701,7 +1701,7 @@
         <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C12" t="s">
         <v>36</v>
@@ -1712,7 +1712,7 @@
         <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
         <v>36</v>
@@ -1723,7 +1723,7 @@
         <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C14" t="s">
         <v>36</v>
@@ -1734,7 +1734,7 @@
         <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C15" t="s">
         <v>36</v>
@@ -1745,13 +1745,13 @@
         <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C16" t="s">
         <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -1759,13 +1759,13 @@
         <v>49</v>
       </c>
       <c r="B17" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C17" t="s">
         <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -1773,13 +1773,13 @@
         <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C18" t="s">
         <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -1787,13 +1787,13 @@
         <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C19" t="s">
         <v>36</v>
       </c>
       <c r="D19" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -1801,13 +1801,13 @@
         <v>52</v>
       </c>
       <c r="B20" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C20" t="s">
         <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -1815,7 +1815,7 @@
         <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C21" t="s">
         <v>36</v>
@@ -1826,7 +1826,7 @@
         <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C22" t="s">
         <v>36</v>
@@ -1837,7 +1837,7 @@
         <v>55</v>
       </c>
       <c r="B23" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C23" t="s">
         <v>36</v>
@@ -1848,7 +1848,7 @@
         <v>56</v>
       </c>
       <c r="B24" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C24" t="s">
         <v>36</v>
@@ -1859,7 +1859,7 @@
         <v>57</v>
       </c>
       <c r="B25" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C25" t="s">
         <v>36</v>
@@ -1881,7 +1881,7 @@
         <v>60</v>
       </c>
       <c r="B27" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C27" t="s">
         <v>36</v>
@@ -1895,7 +1895,7 @@
         <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C28" t="s">
         <v>63</v>
@@ -1909,7 +1909,7 @@
         <v>65</v>
       </c>
       <c r="B29" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C29" t="s">
         <v>63</v>
@@ -1920,7 +1920,7 @@
         <v>66</v>
       </c>
       <c r="B30" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C30" t="s">
         <v>63</v>
@@ -1931,7 +1931,7 @@
         <v>67</v>
       </c>
       <c r="B31" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C31" t="s">
         <v>63</v>
@@ -1942,7 +1942,7 @@
         <v>68</v>
       </c>
       <c r="B32" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C32" t="s">
         <v>63</v>
@@ -1956,7 +1956,7 @@
         <v>70</v>
       </c>
       <c r="B33" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C33" t="s">
         <v>63</v>
@@ -1967,7 +1967,7 @@
         <v>71</v>
       </c>
       <c r="B34" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C34" t="s">
         <v>63</v>
@@ -1978,7 +1978,7 @@
         <v>72</v>
       </c>
       <c r="B35" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C35" t="s">
         <v>63</v>
@@ -1989,10 +1989,10 @@
         <v>73</v>
       </c>
       <c r="B36" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C36" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D36" t="s">
         <v>74</v>
@@ -2003,7 +2003,7 @@
         <v>75</v>
       </c>
       <c r="B37" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C37" t="s">
         <v>33</v>
@@ -2017,10 +2017,10 @@
         <v>77</v>
       </c>
       <c r="B38" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C38" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rename the Bird_abundances metadata sheet to Bird_pcs_all
</commit_message>
<xml_diff>
--- a/DataS1/Column_definitions_final.xlsx
+++ b/DataS1/Column_definitions_final.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ubcca-my.sharepoint.com/personal/aaron_skinner2_ubc_ca/Documents/Academia/PhD/Analysis/Ssp-bird-data-wrangling/DataS1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="11_2A7B806BDA388D21EAE73AD5D10BB879CF387425" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D942B36-CE6E-6646-9D07-396AC5BCF946}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="11_2A7B806BDA388D21EAE73AD5D10BB879CF387425" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94C0018A-6AE8-1D4C-B457-BDCFEEAC2453}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="25120" windowHeight="14840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="25120" windowHeight="14840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Bird_abundances" sheetId="1" r:id="rId1"/>
+    <sheet name="Bird_pcs_all" sheetId="1" r:id="rId1"/>
     <sheet name="Event_covs" sheetId="6" r:id="rId2"/>
     <sheet name="Site_covs" sheetId="3" r:id="rId3"/>
     <sheet name="Functional_traits" sheetId="7" r:id="rId4"/>

</xml_diff>